<commit_message>
Initial commit: NSGA-II & Robin Hood for Exam Scheduling
</commit_message>
<xml_diff>
--- a/data/ca_thi.xlsx
+++ b/data/ca_thi.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,42 +433,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ca thi</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ngày</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>GIỜ</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Thời gian</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Thứ</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>MS Ca thi</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Cơ sở</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Số lượng cán bộ cần thiết</t>
         </is>
@@ -468,7 +480,7 @@
           <t>Thứ 2, 18/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -495,7 +507,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -504,7 +516,7 @@
           <t>Thứ 3, 19/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="2" t="n">
         <v>46161</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -531,7 +543,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -540,7 +552,7 @@
           <t>Thứ 5, 21/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -567,7 +579,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -576,7 +588,7 @@
           <t>Thứ 6, 22/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="2" t="n">
         <v>46164</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -603,7 +615,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -612,7 +624,7 @@
           <t>Thứ 7, 23/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="2" t="n">
         <v>46165</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -639,7 +651,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -648,7 +660,7 @@
           <t>Thứ 2, 25/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" s="2" t="n">
         <v>46167</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -675,7 +687,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -684,7 +696,7 @@
           <t>Thứ 2, 25/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="2" t="n">
         <v>46167</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -711,7 +723,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -720,7 +732,7 @@
           <t>Thứ 3, 26/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="2" t="n">
         <v>46168</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -747,7 +759,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -756,7 +768,7 @@
           <t>Thứ 4, 27/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" s="2" t="n">
         <v>46169</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -783,7 +795,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -792,7 +804,7 @@
           <t>Thứ 4, 27/05/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" s="2" t="n">
         <v>46169</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -828,7 +840,7 @@
           <t>Thứ 4, 27/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B12" s="1" t="n">
+      <c r="B12" s="2" t="n">
         <v>46169</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -855,7 +867,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -864,7 +876,7 @@
           <t>Thứ 5, 28/05/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B13" s="1" t="n">
+      <c r="B13" s="2" t="n">
         <v>46170</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -891,7 +903,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -900,7 +912,7 @@
           <t>Thứ 5, 28/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B14" s="1" t="n">
+      <c r="B14" s="2" t="n">
         <v>46170</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -927,7 +939,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -936,7 +948,7 @@
           <t>Thứ 5, 28/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B15" s="1" t="n">
+      <c r="B15" s="2" t="n">
         <v>46170</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -963,7 +975,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
@@ -972,7 +984,7 @@
           <t>Thứ 5, 28/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B16" s="1" t="n">
+      <c r="B16" s="2" t="n">
         <v>46170</v>
       </c>
       <c r="C16" t="inlineStr">
@@ -1008,7 +1020,7 @@
           <t>Thứ 5, 28/05/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B17" s="1" t="n">
+      <c r="B17" s="2" t="n">
         <v>46170</v>
       </c>
       <c r="C17" t="inlineStr">
@@ -1035,7 +1047,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1044,7 +1056,7 @@
           <t>Thứ 5, 28/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="2" t="n">
         <v>46170</v>
       </c>
       <c r="C18" t="inlineStr">
@@ -1071,7 +1083,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -1080,7 +1092,7 @@
           <t>Thứ 6, 29/05/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B19" s="1" t="n">
+      <c r="B19" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="C19" t="inlineStr">
@@ -1107,7 +1119,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>7</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20">
@@ -1116,7 +1128,7 @@
           <t>Thứ 6, 29/05/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B20" s="1" t="n">
+      <c r="B20" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="C20" t="inlineStr">
@@ -1143,7 +1155,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1152,7 +1164,7 @@
           <t>Thứ 6, 29/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B21" s="1" t="n">
+      <c r="B21" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="C21" t="inlineStr">
@@ -1179,7 +1191,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1188,7 +1200,7 @@
           <t>Thứ 6, 29/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B22" s="1" t="n">
+      <c r="B22" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="C22" t="inlineStr">
@@ -1215,7 +1227,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1224,7 +1236,7 @@
           <t>Thứ 6, 29/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B23" s="1" t="n">
+      <c r="B23" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="C23" t="inlineStr">
@@ -1251,7 +1263,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -1260,7 +1272,7 @@
           <t>Thứ 7, 30/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B24" s="1" t="n">
+      <c r="B24" s="2" t="n">
         <v>46172</v>
       </c>
       <c r="C24" t="inlineStr">
@@ -1287,7 +1299,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -1296,7 +1308,7 @@
           <t>Thứ 7, 30/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B25" s="1" t="n">
+      <c r="B25" s="2" t="n">
         <v>46172</v>
       </c>
       <c r="C25" t="inlineStr">
@@ -1323,7 +1335,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
@@ -1332,7 +1344,7 @@
           <t>Chủ Nhật, 31/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B26" s="1" t="n">
+      <c r="B26" s="2" t="n">
         <v>46173</v>
       </c>
       <c r="C26" t="inlineStr">
@@ -1359,7 +1371,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
@@ -1368,7 +1380,7 @@
           <t>Chủ Nhật, 31/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B27" s="1" t="n">
+      <c r="B27" s="2" t="n">
         <v>46173</v>
       </c>
       <c r="C27" t="inlineStr">
@@ -1395,7 +1407,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28">
@@ -1404,7 +1416,7 @@
           <t>Thứ 2, 01/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B28" s="1" t="n">
+      <c r="B28" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="C28" t="inlineStr">
@@ -1431,7 +1443,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1440,7 +1452,7 @@
           <t>Thứ 2, 01/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B29" s="1" t="n">
+      <c r="B29" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="C29" t="inlineStr">
@@ -1467,7 +1479,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30">
@@ -1476,7 +1488,7 @@
           <t>Thứ 2, 01/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B30" s="1" t="n">
+      <c r="B30" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="C30" t="inlineStr">
@@ -1503,7 +1515,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>5</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31">
@@ -1512,7 +1524,7 @@
           <t>Thứ 2, 01/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B31" s="1" t="n">
+      <c r="B31" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="C31" t="inlineStr">
@@ -1539,7 +1551,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -1548,7 +1560,7 @@
           <t>Thứ 2, 01/06/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B32" s="1" t="n">
+      <c r="B32" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="C32" t="inlineStr">
@@ -1575,7 +1587,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -1584,7 +1596,7 @@
           <t>Thứ 3, 02/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B33" s="1" t="n">
+      <c r="B33" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="C33" t="inlineStr">
@@ -1611,7 +1623,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -1620,7 +1632,7 @@
           <t>Thứ 3, 02/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B34" s="1" t="n">
+      <c r="B34" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="C34" t="inlineStr">
@@ -1647,7 +1659,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35">
@@ -1656,7 +1668,7 @@
           <t>Thứ 3, 02/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B35" s="1" t="n">
+      <c r="B35" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="C35" t="inlineStr">
@@ -1683,7 +1695,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
     <row r="36">
@@ -1692,7 +1704,7 @@
           <t>Thứ 3, 02/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B36" s="1" t="n">
+      <c r="B36" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="C36" t="inlineStr">
@@ -1719,7 +1731,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37">
@@ -1728,7 +1740,7 @@
           <t>Thứ 3, 02/06/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B37" s="1" t="n">
+      <c r="B37" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="C37" t="inlineStr">
@@ -1755,7 +1767,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -1764,7 +1776,7 @@
           <t>Thứ 4, 03/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B38" s="1" t="n">
+      <c r="B38" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="C38" t="inlineStr">
@@ -1791,7 +1803,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39">
@@ -1800,7 +1812,7 @@
           <t>Thứ 4, 03/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B39" s="1" t="n">
+      <c r="B39" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="C39" t="inlineStr">
@@ -1827,7 +1839,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
     </row>
     <row r="40">
@@ -1836,7 +1848,7 @@
           <t>Thứ 4, 03/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B40" s="1" t="n">
+      <c r="B40" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="C40" t="inlineStr">
@@ -1863,7 +1875,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>7</v>
+        <v>31</v>
       </c>
     </row>
     <row r="41">
@@ -1872,7 +1884,7 @@
           <t>Thứ 4, 03/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B41" s="1" t="n">
+      <c r="B41" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="C41" t="inlineStr">
@@ -1899,7 +1911,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="42">
@@ -1908,7 +1920,7 @@
           <t>Thứ 5, 04/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B42" s="1" t="n">
+      <c r="B42" s="2" t="n">
         <v>46177</v>
       </c>
       <c r="C42" t="inlineStr">
@@ -1935,7 +1947,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43">
@@ -1944,7 +1956,7 @@
           <t>Thứ 5, 04/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B43" s="1" t="n">
+      <c r="B43" s="2" t="n">
         <v>46177</v>
       </c>
       <c r="C43" t="inlineStr">
@@ -1971,7 +1983,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44">
@@ -1980,7 +1992,7 @@
           <t>Thứ 5, 04/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B44" s="1" t="n">
+      <c r="B44" s="2" t="n">
         <v>46177</v>
       </c>
       <c r="C44" t="inlineStr">
@@ -2007,7 +2019,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="45">
@@ -2016,7 +2028,7 @@
           <t>Thứ 5, 04/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B45" s="1" t="n">
+      <c r="B45" s="2" t="n">
         <v>46177</v>
       </c>
       <c r="C45" t="inlineStr">
@@ -2043,7 +2055,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -2052,7 +2064,7 @@
           <t>Thứ 6, 05/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B46" s="1" t="n">
+      <c r="B46" s="2" t="n">
         <v>46178</v>
       </c>
       <c r="C46" t="inlineStr">
@@ -2079,7 +2091,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="47">
@@ -2088,7 +2100,7 @@
           <t>Thứ 6, 05/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B47" s="1" t="n">
+      <c r="B47" s="2" t="n">
         <v>46178</v>
       </c>
       <c r="C47" t="inlineStr">
@@ -2115,7 +2127,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="48">
@@ -2124,7 +2136,7 @@
           <t>Thứ 6, 05/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B48" s="1" t="n">
+      <c r="B48" s="2" t="n">
         <v>46178</v>
       </c>
       <c r="C48" t="inlineStr">
@@ -2151,7 +2163,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="49">
@@ -2160,7 +2172,7 @@
           <t>Thứ 2, 08/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B49" s="1" t="n">
+      <c r="B49" s="2" t="n">
         <v>46181</v>
       </c>
       <c r="C49" t="inlineStr">
@@ -2187,7 +2199,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50">
@@ -2196,7 +2208,7 @@
           <t>Thứ 2, 08/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B50" s="1" t="n">
+      <c r="B50" s="2" t="n">
         <v>46181</v>
       </c>
       <c r="C50" t="inlineStr">
@@ -2223,7 +2235,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="51">
@@ -2232,7 +2244,7 @@
           <t>Thứ 2, 08/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B51" s="1" t="n">
+      <c r="B51" s="2" t="n">
         <v>46181</v>
       </c>
       <c r="C51" t="inlineStr">
@@ -2259,7 +2271,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -2268,7 +2280,7 @@
           <t>Thứ 3, 09/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B52" s="1" t="n">
+      <c r="B52" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="C52" t="inlineStr">
@@ -2295,7 +2307,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="53">
@@ -2304,7 +2316,7 @@
           <t>Thứ 3, 09/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B53" s="1" t="n">
+      <c r="B53" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="C53" t="inlineStr">
@@ -2331,7 +2343,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54">
@@ -2340,7 +2352,7 @@
           <t>Thứ 3, 09/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B54" s="1" t="n">
+      <c r="B54" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="C54" t="inlineStr">
@@ -2367,7 +2379,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="55">
@@ -2376,7 +2388,7 @@
           <t>Thứ 4, 10/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B55" s="1" t="n">
+      <c r="B55" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="C55" t="inlineStr">
@@ -2403,7 +2415,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="56">
@@ -2412,7 +2424,7 @@
           <t>Thứ 4, 10/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B56" s="1" t="n">
+      <c r="B56" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="C56" t="inlineStr">
@@ -2448,7 +2460,7 @@
           <t>Thứ 5, 11/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B57" s="1" t="n">
+      <c r="B57" s="2" t="n">
         <v>46184</v>
       </c>
       <c r="C57" t="inlineStr">
@@ -2475,7 +2487,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
     </row>
     <row r="58">
@@ -2484,7 +2496,7 @@
           <t>Thứ 5, 11/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B58" s="1" t="n">
+      <c r="B58" s="2" t="n">
         <v>46184</v>
       </c>
       <c r="C58" t="inlineStr">
@@ -2511,7 +2523,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
@@ -2520,7 +2532,7 @@
           <t>Thứ 6, 12/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B59" s="1" t="n">
+      <c r="B59" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="C59" t="inlineStr">
@@ -2547,7 +2559,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
     </row>
     <row r="60">
@@ -2556,7 +2568,7 @@
           <t>Thứ 6, 12/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B60" s="1" t="n">
+      <c r="B60" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="C60" t="inlineStr">
@@ -2583,7 +2595,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61">
@@ -2592,7 +2604,7 @@
           <t>Thứ 6, 12/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B61" s="1" t="n">
+      <c r="B61" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="C61" t="inlineStr">
@@ -2619,7 +2631,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
     </row>
     <row r="62">
@@ -2628,7 +2640,7 @@
           <t>Thứ 6, 12/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B62" s="1" t="n">
+      <c r="B62" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="C62" t="inlineStr">
@@ -2655,7 +2667,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
     </row>
     <row r="63">
@@ -2664,7 +2676,7 @@
           <t>Thứ 7, 13/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B63" s="1" t="n">
+      <c r="B63" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="C63" t="inlineStr">
@@ -2700,7 +2712,7 @@
           <t>Thứ 7, 13/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B64" s="1" t="n">
+      <c r="B64" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="C64" t="inlineStr">
@@ -2727,7 +2739,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="65">
@@ -2736,7 +2748,7 @@
           <t>Thứ 7, 13/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B65" s="1" t="n">
+      <c r="B65" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="C65" t="inlineStr">
@@ -2763,7 +2775,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
@@ -2772,7 +2784,7 @@
           <t>Thứ 7, 13/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B66" s="1" t="n">
+      <c r="B66" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="C66" t="inlineStr">
@@ -2799,7 +2811,7 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67">
@@ -2808,7 +2820,7 @@
           <t>Thứ 7, 13/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B67" s="1" t="n">
+      <c r="B67" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="C67" t="inlineStr">
@@ -2835,7 +2847,7 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="68">
@@ -2844,7 +2856,7 @@
           <t>Thứ 7, 13/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B68" s="1" t="n">
+      <c r="B68" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="C68" t="inlineStr">
@@ -2871,7 +2883,7 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69">
@@ -2880,7 +2892,7 @@
           <t>Thứ 7, 13/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B69" s="1" t="n">
+      <c r="B69" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="C69" t="inlineStr">
@@ -2907,7 +2919,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70">
@@ -2916,7 +2928,7 @@
           <t>Thứ 2, 08/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B70" s="1" t="n">
+      <c r="B70" s="2" t="n">
         <v>46181</v>
       </c>
       <c r="C70" t="inlineStr">
@@ -2943,7 +2955,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
@@ -2952,7 +2964,7 @@
           <t>Thứ 2, 08/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B71" s="1" t="n">
+      <c r="B71" s="2" t="n">
         <v>46181</v>
       </c>
       <c r="C71" t="inlineStr">
@@ -2979,7 +2991,7 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
@@ -2988,7 +3000,7 @@
           <t>Thứ 2, 08/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B72" s="1" t="n">
+      <c r="B72" s="2" t="n">
         <v>46181</v>
       </c>
       <c r="C72" t="inlineStr">
@@ -3024,7 +3036,7 @@
           <t>Thứ 2, 08/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B73" s="1" t="n">
+      <c r="B73" s="2" t="n">
         <v>46181</v>
       </c>
       <c r="C73" t="inlineStr">
@@ -3051,7 +3063,7 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74">
@@ -3060,7 +3072,7 @@
           <t>Thứ 3, 09/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B74" s="1" t="n">
+      <c r="B74" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="C74" t="inlineStr">
@@ -3087,7 +3099,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -3096,7 +3108,7 @@
           <t>Thứ 4, 10/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B75" s="1" t="n">
+      <c r="B75" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="C75" t="inlineStr">
@@ -3123,7 +3135,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -3132,7 +3144,7 @@
           <t>Thứ 4, 10/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B76" s="1" t="n">
+      <c r="B76" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="C76" t="inlineStr">
@@ -3159,7 +3171,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -3168,7 +3180,7 @@
           <t>Thứ 4, 10/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B77" s="1" t="n">
+      <c r="B77" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="C77" t="inlineStr">
@@ -3195,7 +3207,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -3204,7 +3216,7 @@
           <t>Thứ 4, 10/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B78" s="1" t="n">
+      <c r="B78" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="C78" t="inlineStr">
@@ -3231,7 +3243,7 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -3240,7 +3252,7 @@
           <t>Thứ 5, 11/06/2026, Ca1 : 07g00-09g30</t>
         </is>
       </c>
-      <c r="B79" s="1" t="n">
+      <c r="B79" s="2" t="n">
         <v>46184</v>
       </c>
       <c r="C79" t="inlineStr">
@@ -3267,7 +3279,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -3276,7 +3288,7 @@
           <t>Thứ 6, 12/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B80" s="1" t="n">
+      <c r="B80" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="C80" t="inlineStr">
@@ -3303,7 +3315,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81">
@@ -3312,7 +3324,7 @@
           <t>Thứ 6, 12/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B81" s="1" t="n">
+      <c r="B81" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="C81" t="inlineStr">
@@ -3339,7 +3351,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update config by 3T
</commit_message>
<xml_diff>
--- a/data/ca_thi.xlsx
+++ b/data/ca_thi.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,42 +421,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ca thi</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ngày</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>GIỜ</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Thời gian</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Thứ</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>MS Ca thi</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Cơ sở</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Số lượng cán bộ cần thiết</t>
         </is>
@@ -480,7 +468,7 @@
           <t>Thứ 2, 18/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -507,7 +495,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -516,7 +504,7 @@
           <t>Thứ 3, 19/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -543,7 +531,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -552,7 +540,7 @@
           <t>Thứ 5, 21/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="1" t="n">
         <v>46163</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -579,7 +567,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -588,7 +576,7 @@
           <t>Thứ 6, 22/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="1" t="n">
         <v>46164</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -615,7 +603,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -624,7 +612,7 @@
           <t>Thứ 7, 23/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="1" t="n">
         <v>46165</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -651,7 +639,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -660,7 +648,7 @@
           <t>Thứ 2, 25/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -687,7 +675,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -696,7 +684,7 @@
           <t>Thứ 2, 25/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -723,7 +711,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -732,7 +720,7 @@
           <t>Thứ 3, 26/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="1" t="n">
         <v>46168</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -759,7 +747,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -768,7 +756,7 @@
           <t>Thứ 4, 27/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="1" t="n">
         <v>46169</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -795,7 +783,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -804,7 +792,7 @@
           <t>Thứ 4, 27/05/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="1" t="n">
         <v>46169</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -840,7 +828,7 @@
           <t>Thứ 4, 27/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="1" t="n">
         <v>46169</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -867,7 +855,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -876,7 +864,7 @@
           <t>Thứ 5, 28/05/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -903,7 +891,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -912,7 +900,7 @@
           <t>Thứ 5, 28/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -939,7 +927,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -948,7 +936,7 @@
           <t>Thứ 5, 28/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -975,7 +963,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -984,7 +972,7 @@
           <t>Thứ 5, 28/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="C16" t="inlineStr">
@@ -1020,7 +1008,7 @@
           <t>Thứ 5, 28/05/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="C17" t="inlineStr">
@@ -1047,7 +1035,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
@@ -1056,7 +1044,7 @@
           <t>Thứ 5, 28/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B18" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="C18" t="inlineStr">
@@ -1083,7 +1071,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -1092,7 +1080,7 @@
           <t>Thứ 6, 29/05/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="C19" t="inlineStr">
@@ -1119,7 +1107,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -1128,7 +1116,7 @@
           <t>Thứ 6, 29/05/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="C20" t="inlineStr">
@@ -1155,7 +1143,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -1164,7 +1152,7 @@
           <t>Thứ 6, 29/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B21" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="C21" t="inlineStr">
@@ -1191,7 +1179,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22">
@@ -1200,7 +1188,7 @@
           <t>Thứ 6, 29/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B22" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="C22" t="inlineStr">
@@ -1227,7 +1215,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
@@ -1236,7 +1224,7 @@
           <t>Thứ 6, 29/05/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B23" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="C23" t="inlineStr">
@@ -1263,7 +1251,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1272,7 +1260,7 @@
           <t>Thứ 7, 30/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B24" s="1" t="n">
         <v>46172</v>
       </c>
       <c r="C24" t="inlineStr">
@@ -1299,7 +1287,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -1308,7 +1296,7 @@
           <t>Thứ 7, 30/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B25" s="1" t="n">
         <v>46172</v>
       </c>
       <c r="C25" t="inlineStr">
@@ -1335,7 +1323,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
@@ -1344,7 +1332,7 @@
           <t>Chủ Nhật, 31/05/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B26" s="1" t="n">
         <v>46173</v>
       </c>
       <c r="C26" t="inlineStr">
@@ -1371,7 +1359,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -1380,7 +1368,7 @@
           <t>Chủ Nhật, 31/05/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B27" s="1" t="n">
         <v>46173</v>
       </c>
       <c r="C27" t="inlineStr">
@@ -1407,7 +1395,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -1416,7 +1404,7 @@
           <t>Thứ 2, 01/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B28" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C28" t="inlineStr">
@@ -1443,7 +1431,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -1452,7 +1440,7 @@
           <t>Thứ 2, 01/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B29" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C29" t="inlineStr">
@@ -1479,7 +1467,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -1488,7 +1476,7 @@
           <t>Thứ 2, 01/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B30" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C30" t="inlineStr">
@@ -1515,7 +1503,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31">
@@ -1524,7 +1512,7 @@
           <t>Thứ 2, 01/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B31" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C31" t="inlineStr">
@@ -1551,7 +1539,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32">
@@ -1560,7 +1548,7 @@
           <t>Thứ 2, 01/06/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B32" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C32" t="inlineStr">
@@ -1587,7 +1575,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33">
@@ -1596,7 +1584,7 @@
           <t>Thứ 3, 02/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
+      <c r="B33" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="C33" t="inlineStr">
@@ -1623,7 +1611,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
@@ -1632,7 +1620,7 @@
           <t>Thứ 3, 02/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B34" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="C34" t="inlineStr">
@@ -1659,7 +1647,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -1668,7 +1656,7 @@
           <t>Thứ 3, 02/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B35" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="C35" t="inlineStr">
@@ -1695,7 +1683,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -1704,7 +1692,7 @@
           <t>Thứ 3, 02/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B36" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="C36" t="inlineStr">
@@ -1731,7 +1719,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37">
@@ -1740,7 +1728,7 @@
           <t>Thứ 3, 02/06/2026, Ca 5: 18g15-20g45</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B37" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="C37" t="inlineStr">
@@ -1767,7 +1755,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
@@ -1776,7 +1764,7 @@
           <t>Thứ 4, 03/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
+      <c r="B38" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="C38" t="inlineStr">
@@ -1803,7 +1791,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>31</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39">
@@ -1812,7 +1800,7 @@
           <t>Thứ 4, 03/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
+      <c r="B39" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="C39" t="inlineStr">
@@ -1839,7 +1827,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
@@ -1848,7 +1836,7 @@
           <t>Thứ 4, 03/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
+      <c r="B40" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="C40" t="inlineStr">
@@ -1875,7 +1863,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41">
@@ -1884,7 +1872,7 @@
           <t>Thứ 4, 03/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B41" s="2" t="n">
+      <c r="B41" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="C41" t="inlineStr">
@@ -1911,7 +1899,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -1920,7 +1908,7 @@
           <t>Thứ 5, 04/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n">
+      <c r="B42" s="1" t="n">
         <v>46177</v>
       </c>
       <c r="C42" t="inlineStr">
@@ -1947,7 +1935,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -1956,7 +1944,7 @@
           <t>Thứ 5, 04/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B43" s="1" t="n">
         <v>46177</v>
       </c>
       <c r="C43" t="inlineStr">
@@ -1983,7 +1971,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44">
@@ -1992,7 +1980,7 @@
           <t>Thứ 5, 04/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
+      <c r="B44" s="1" t="n">
         <v>46177</v>
       </c>
       <c r="C44" t="inlineStr">
@@ -2019,7 +2007,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45">
@@ -2028,7 +2016,7 @@
           <t>Thứ 5, 04/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B45" s="2" t="n">
+      <c r="B45" s="1" t="n">
         <v>46177</v>
       </c>
       <c r="C45" t="inlineStr">
@@ -2055,7 +2043,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -2064,7 +2052,7 @@
           <t>Thứ 6, 05/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n">
+      <c r="B46" s="1" t="n">
         <v>46178</v>
       </c>
       <c r="C46" t="inlineStr">
@@ -2091,7 +2079,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47">
@@ -2100,7 +2088,7 @@
           <t>Thứ 6, 05/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B47" s="2" t="n">
+      <c r="B47" s="1" t="n">
         <v>46178</v>
       </c>
       <c r="C47" t="inlineStr">
@@ -2127,7 +2115,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48">
@@ -2136,7 +2124,7 @@
           <t>Thứ 6, 05/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B48" s="2" t="n">
+      <c r="B48" s="1" t="n">
         <v>46178</v>
       </c>
       <c r="C48" t="inlineStr">
@@ -2163,7 +2151,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49">
@@ -2172,7 +2160,7 @@
           <t>Thứ 2, 08/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B49" s="2" t="n">
+      <c r="B49" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="C49" t="inlineStr">
@@ -2199,7 +2187,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -2208,7 +2196,7 @@
           <t>Thứ 2, 08/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B50" s="2" t="n">
+      <c r="B50" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="C50" t="inlineStr">
@@ -2235,7 +2223,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51">
@@ -2244,7 +2232,7 @@
           <t>Thứ 2, 08/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B51" s="2" t="n">
+      <c r="B51" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="C51" t="inlineStr">
@@ -2271,7 +2259,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52">
@@ -2280,7 +2268,7 @@
           <t>Thứ 3, 09/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B52" s="2" t="n">
+      <c r="B52" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="C52" t="inlineStr">
@@ -2307,7 +2295,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53">
@@ -2316,7 +2304,7 @@
           <t>Thứ 3, 09/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B53" s="2" t="n">
+      <c r="B53" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="C53" t="inlineStr">
@@ -2343,7 +2331,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
@@ -2352,7 +2340,7 @@
           <t>Thứ 3, 09/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B54" s="2" t="n">
+      <c r="B54" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="C54" t="inlineStr">
@@ -2379,7 +2367,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55">
@@ -2388,7 +2376,7 @@
           <t>Thứ 4, 10/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B55" s="2" t="n">
+      <c r="B55" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="C55" t="inlineStr">
@@ -2415,7 +2403,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -2424,7 +2412,7 @@
           <t>Thứ 4, 10/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B56" s="2" t="n">
+      <c r="B56" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="C56" t="inlineStr">
@@ -2460,7 +2448,7 @@
           <t>Thứ 5, 11/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B57" s="2" t="n">
+      <c r="B57" s="1" t="n">
         <v>46184</v>
       </c>
       <c r="C57" t="inlineStr">
@@ -2487,7 +2475,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
     </row>
     <row r="58">
@@ -2496,7 +2484,7 @@
           <t>Thứ 5, 11/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B58" s="2" t="n">
+      <c r="B58" s="1" t="n">
         <v>46184</v>
       </c>
       <c r="C58" t="inlineStr">
@@ -2523,7 +2511,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -2532,7 +2520,7 @@
           <t>Thứ 6, 12/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B59" s="2" t="n">
+      <c r="B59" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="C59" t="inlineStr">
@@ -2559,7 +2547,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
@@ -2568,7 +2556,7 @@
           <t>Thứ 6, 12/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B60" s="2" t="n">
+      <c r="B60" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="C60" t="inlineStr">
@@ -2595,7 +2583,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="61">
@@ -2604,7 +2592,7 @@
           <t>Thứ 6, 12/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B61" s="2" t="n">
+      <c r="B61" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="C61" t="inlineStr">
@@ -2631,7 +2619,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62">
@@ -2640,7 +2628,7 @@
           <t>Thứ 6, 12/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B62" s="2" t="n">
+      <c r="B62" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="C62" t="inlineStr">
@@ -2667,7 +2655,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63">
@@ -2676,7 +2664,7 @@
           <t>Thứ 7, 13/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B63" s="2" t="n">
+      <c r="B63" s="1" t="n">
         <v>46186</v>
       </c>
       <c r="C63" t="inlineStr">
@@ -2712,7 +2700,7 @@
           <t>Thứ 7, 13/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B64" s="2" t="n">
+      <c r="B64" s="1" t="n">
         <v>46186</v>
       </c>
       <c r="C64" t="inlineStr">
@@ -2739,7 +2727,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65">
@@ -2748,7 +2736,7 @@
           <t>Thứ 7, 13/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B65" s="2" t="n">
+      <c r="B65" s="1" t="n">
         <v>46186</v>
       </c>
       <c r="C65" t="inlineStr">
@@ -2775,7 +2763,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -2784,7 +2772,7 @@
           <t>Thứ 7, 13/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B66" s="2" t="n">
+      <c r="B66" s="1" t="n">
         <v>46186</v>
       </c>
       <c r="C66" t="inlineStr">
@@ -2811,7 +2799,7 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="67">
@@ -2820,7 +2808,7 @@
           <t>Thứ 7, 13/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B67" s="2" t="n">
+      <c r="B67" s="1" t="n">
         <v>46186</v>
       </c>
       <c r="C67" t="inlineStr">
@@ -2847,7 +2835,7 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="68">
@@ -2856,7 +2844,7 @@
           <t>Thứ 7, 13/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B68" s="2" t="n">
+      <c r="B68" s="1" t="n">
         <v>46186</v>
       </c>
       <c r="C68" t="inlineStr">
@@ -2883,7 +2871,7 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -2892,7 +2880,7 @@
           <t>Thứ 7, 13/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B69" s="2" t="n">
+      <c r="B69" s="1" t="n">
         <v>46186</v>
       </c>
       <c r="C69" t="inlineStr">
@@ -2919,7 +2907,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -2928,7 +2916,7 @@
           <t>Thứ 2, 08/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B70" s="2" t="n">
+      <c r="B70" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="C70" t="inlineStr">
@@ -2955,7 +2943,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="71">
@@ -2964,7 +2952,7 @@
           <t>Thứ 2, 08/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B71" s="2" t="n">
+      <c r="B71" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="C71" t="inlineStr">
@@ -2991,7 +2979,7 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
@@ -3000,7 +2988,7 @@
           <t>Thứ 2, 08/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B72" s="2" t="n">
+      <c r="B72" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="C72" t="inlineStr">
@@ -3036,7 +3024,7 @@
           <t>Thứ 2, 08/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B73" s="2" t="n">
+      <c r="B73" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="C73" t="inlineStr">
@@ -3063,7 +3051,7 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74">
@@ -3072,7 +3060,7 @@
           <t>Thứ 3, 09/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B74" s="2" t="n">
+      <c r="B74" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="C74" t="inlineStr">
@@ -3099,7 +3087,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75">
@@ -3108,7 +3096,7 @@
           <t>Thứ 4, 10/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B75" s="2" t="n">
+      <c r="B75" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="C75" t="inlineStr">
@@ -3135,7 +3123,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76">
@@ -3144,7 +3132,7 @@
           <t>Thứ 4, 10/06/2026, Ca 1: 07g00-09g30</t>
         </is>
       </c>
-      <c r="B76" s="2" t="n">
+      <c r="B76" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="C76" t="inlineStr">
@@ -3171,7 +3159,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="77">
@@ -3180,7 +3168,7 @@
           <t>Thứ 4, 10/06/2026, Ca 2: 09g30-12g00</t>
         </is>
       </c>
-      <c r="B77" s="2" t="n">
+      <c r="B77" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="C77" t="inlineStr">
@@ -3207,7 +3195,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78">
@@ -3216,7 +3204,7 @@
           <t>Thứ 4, 10/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B78" s="2" t="n">
+      <c r="B78" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="C78" t="inlineStr">
@@ -3243,7 +3231,7 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79">
@@ -3252,7 +3240,7 @@
           <t>Thứ 5, 11/06/2026, Ca1 : 07g00-09g30</t>
         </is>
       </c>
-      <c r="B79" s="2" t="n">
+      <c r="B79" s="1" t="n">
         <v>46184</v>
       </c>
       <c r="C79" t="inlineStr">
@@ -3279,7 +3267,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="80">
@@ -3288,7 +3276,7 @@
           <t>Thứ 6, 12/06/2026, Ca 3: 13g00-15g30</t>
         </is>
       </c>
-      <c r="B80" s="2" t="n">
+      <c r="B80" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="C80" t="inlineStr">
@@ -3315,7 +3303,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -3324,7 +3312,7 @@
           <t>Thứ 6, 12/06/2026, Ca 4: 15g30-18g00</t>
         </is>
       </c>
-      <c r="B81" s="2" t="n">
+      <c r="B81" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="C81" t="inlineStr">
@@ -3351,7 +3339,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>